<commit_message>
clean sumo test data
</commit_message>
<xml_diff>
--- a/assets/raw-data/sumo/cc2_feat_projection_v3.0.3.xlsx
+++ b/assets/raw-data/sumo/cc2_feat_projection_v3.0.3.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="20402"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="20415"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DrebenstedtN\mex-extractors\assets\raw-data\sumo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HesseE\mex-extractors\assets\raw-data\sumo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E4A4D5E-2859-4B1E-8B2E-7558D89F99AB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6FAF9DA-CEE0-4191-8E3D-5A0EC413B0D3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="12">
   <si>
     <r>
       <t>feature</t>
@@ -127,37 +127,13 @@
     <t>RSV</t>
   </si>
   <si>
-    <t>respiratory syncytial virus, specific</t>
-  </si>
-  <si>
-    <t>Respiratorisches Syncytial-Virus, spezifisch</t>
-  </si>
-  <si>
-    <t>specific RSV-ICD-10 codes</t>
-  </si>
-  <si>
-    <t>respiratory syncytial virus, unspecific</t>
-  </si>
-  <si>
-    <t>Respiratorisches Syncytial-Virus, unspezifisch</t>
-  </si>
-  <si>
-    <t>unspecific ALRI-ICD-10 codes AND &lt;=2 years old</t>
-  </si>
-  <si>
     <t>GI</t>
   </si>
   <si>
-    <t>non-bleeding unspecific gastrointestinal infections</t>
+    <t/>
   </si>
   <si>
-    <t>nicht-blutige unspezifische gastrointestinale Infektionen</t>
-  </si>
-  <si>
-    <t>MTS/CEDIS + gi-specific ICD (non bloody)</t>
-  </si>
-  <si>
-    <t/>
+    <t>Lorem Ipsum</t>
   </si>
 </sst>
 </file>
@@ -281,7 +257,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -300,9 +276,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -319,7 +292,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -623,16 +596,16 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:AD16"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.28515625" style="12" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.7109375" style="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.5703125" style="13" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="39.28515625" style="12" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="76.5703125" style="12" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="60.5703125" style="12" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="82.5703125" style="14" bestFit="1" customWidth="1"/>
-    <col min="8" max="30" width="13.5703125" style="12" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.28515625" style="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.7109375" style="11" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.5703125" style="12" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="39.28515625" style="11" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="76.5703125" style="11" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="60.5703125" style="11" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="82.5703125" style="13" bestFit="1" customWidth="1"/>
+    <col min="8" max="30" width="13.5703125" style="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:30" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -696,12 +669,12 @@
         <v>feat_syndrome_RSV_01</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="G2" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" s="11" t="s">
         <v>11</v>
       </c>
       <c r="H2" s="5"/>
@@ -742,14 +715,14 @@
         <f>A3&amp;"_"&amp;B3&amp;"_"&amp;TEXT(C3,"00")</f>
         <v>feat_syndrome_RSV_02</v>
       </c>
-      <c r="E3" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G3" s="8" t="s">
-        <v>14</v>
+      <c r="E3" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>11</v>
       </c>
       <c r="H3" s="5"/>
       <c r="I3" s="5"/>
@@ -780,7 +753,7 @@
         <v>7</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="C4" s="6">
         <v>1</v>
@@ -789,14 +762,14 @@
         <f>A4&amp;"_"&amp;B4&amp;"_"&amp;TEXT(C4,"00")</f>
         <v>feat_syndrome_GI_01</v>
       </c>
-      <c r="E4" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G4" s="8" t="s">
-        <v>18</v>
+      <c r="E4" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>11</v>
       </c>
       <c r="H4" s="5"/>
       <c r="I4" s="5"/>
@@ -823,24 +796,24 @@
       <c r="AD4" s="5"/>
     </row>
     <row r="5" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A5" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>19</v>
+      <c r="A5" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>10</v>
       </c>
       <c r="C5" s="6"/>
-      <c r="D5" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E5" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F5" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="G5" s="10" t="s">
-        <v>19</v>
+      <c r="D5" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>10</v>
       </c>
       <c r="H5" s="5"/>
       <c r="I5" s="5"/>
@@ -867,24 +840,24 @@
       <c r="AD5" s="5"/>
     </row>
     <row r="6" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A6" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>19</v>
+      <c r="A6" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>10</v>
       </c>
       <c r="C6" s="6"/>
-      <c r="D6" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="G6" s="10" t="s">
-        <v>19</v>
+      <c r="D6" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>10</v>
       </c>
       <c r="H6" s="5"/>
       <c r="I6" s="5"/>
@@ -911,24 +884,24 @@
       <c r="AD6" s="5"/>
     </row>
     <row r="7" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A7" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>19</v>
+      <c r="A7" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>10</v>
       </c>
       <c r="C7" s="6"/>
-      <c r="D7" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F7" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="G7" s="10" t="s">
-        <v>19</v>
+      <c r="D7" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>10</v>
       </c>
       <c r="H7" s="5"/>
       <c r="I7" s="5"/>
@@ -955,24 +928,24 @@
       <c r="AD7" s="5"/>
     </row>
     <row r="8" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A8" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>19</v>
+      <c r="A8" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>10</v>
       </c>
       <c r="C8" s="6"/>
-      <c r="D8" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E8" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F8" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="G8" s="10" t="s">
-        <v>19</v>
+      <c r="D8" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>10</v>
       </c>
       <c r="H8" s="5"/>
       <c r="I8" s="5"/>
@@ -999,24 +972,24 @@
       <c r="AD8" s="5"/>
     </row>
     <row r="9" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A9" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>19</v>
+      <c r="A9" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>10</v>
       </c>
       <c r="C9" s="6"/>
-      <c r="D9" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E9" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F9" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="G9" s="10" t="s">
-        <v>19</v>
+      <c r="D9" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G9" s="9" t="s">
+        <v>10</v>
       </c>
       <c r="H9" s="5"/>
       <c r="I9" s="5"/>
@@ -1043,24 +1016,24 @@
       <c r="AD9" s="5"/>
     </row>
     <row r="10" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A10" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>19</v>
+      <c r="A10" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>10</v>
       </c>
       <c r="C10" s="6"/>
-      <c r="D10" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F10" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="G10" s="10" t="s">
-        <v>19</v>
+      <c r="D10" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G10" s="9" t="s">
+        <v>10</v>
       </c>
       <c r="H10" s="5"/>
       <c r="I10" s="5"/>
@@ -1087,24 +1060,24 @@
       <c r="AD10" s="5"/>
     </row>
     <row r="11" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A11" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>19</v>
+      <c r="A11" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>10</v>
       </c>
       <c r="C11" s="6"/>
-      <c r="D11" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E11" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F11" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="G11" s="10" t="s">
-        <v>19</v>
+      <c r="D11" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G11" s="9" t="s">
+        <v>10</v>
       </c>
       <c r="H11" s="5"/>
       <c r="I11" s="5"/>
@@ -1131,24 +1104,24 @@
       <c r="AD11" s="5"/>
     </row>
     <row r="12" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A12" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>19</v>
+      <c r="A12" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>10</v>
       </c>
       <c r="C12" s="6"/>
-      <c r="D12" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E12" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F12" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="G12" s="10" t="s">
-        <v>19</v>
+      <c r="D12" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G12" s="9" t="s">
+        <v>10</v>
       </c>
       <c r="H12" s="5"/>
       <c r="I12" s="5"/>
@@ -1175,24 +1148,24 @@
       <c r="AD12" s="5"/>
     </row>
     <row r="13" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A13" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>19</v>
+      <c r="A13" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>10</v>
       </c>
       <c r="C13" s="6"/>
-      <c r="D13" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E13" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F13" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="G13" s="10" t="s">
-        <v>19</v>
+      <c r="D13" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G13" s="9" t="s">
+        <v>10</v>
       </c>
       <c r="H13" s="5"/>
       <c r="I13" s="5"/>
@@ -1219,24 +1192,24 @@
       <c r="AD13" s="5"/>
     </row>
     <row r="14" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A14" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B14" s="9" t="s">
-        <v>19</v>
+      <c r="A14" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>10</v>
       </c>
       <c r="C14" s="6"/>
-      <c r="D14" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E14" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F14" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="G14" s="10" t="s">
-        <v>19</v>
+      <c r="D14" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G14" s="9" t="s">
+        <v>10</v>
       </c>
       <c r="H14" s="5"/>
       <c r="I14" s="5"/>
@@ -1263,24 +1236,24 @@
       <c r="AD14" s="5"/>
     </row>
     <row r="15" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A15" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B15" s="9" t="s">
-        <v>19</v>
+      <c r="A15" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>10</v>
       </c>
       <c r="C15" s="6"/>
-      <c r="D15" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E15" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F15" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="G15" s="10" t="s">
-        <v>19</v>
+      <c r="D15" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G15" s="9" t="s">
+        <v>10</v>
       </c>
       <c r="H15" s="5"/>
       <c r="I15" s="5"/>
@@ -1307,24 +1280,24 @@
       <c r="AD15" s="5"/>
     </row>
     <row r="16" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A16" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B16" s="9" t="s">
-        <v>19</v>
+      <c r="A16" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>10</v>
       </c>
       <c r="C16" s="6"/>
-      <c r="D16" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E16" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F16" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="G16" s="11" t="s">
-        <v>19</v>
+      <c r="D16" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G16" s="10" t="s">
+        <v>10</v>
       </c>
       <c r="H16" s="5"/>
       <c r="I16" s="5"/>

</xml_diff>

<commit_message>
Feature/mx 1705 clean up test data (#342)
### Changes
- update test mappings
- update seqrepo, odk, datschaweb, sumo, synopse test data

---------

Signed-off-by: erichesse <eric.hesse3@yahoo.de>
Signed-off-by: erichesse <hessee@rki.de>
Co-authored-by: Franziska Diehr <DiehrF@rki.de>
Co-authored-by: Nicolas Drebenstedt <897972+cutoffthetop@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/assets/raw-data/sumo/cc2_feat_projection_v3.0.3.xlsx
+++ b/assets/raw-data/sumo/cc2_feat_projection_v3.0.3.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="20402"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="20415"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DrebenstedtN\mex-extractors\assets\raw-data\sumo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HesseE\mex-extractors\assets\raw-data\sumo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E4A4D5E-2859-4B1E-8B2E-7558D89F99AB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6FAF9DA-CEE0-4191-8E3D-5A0EC413B0D3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="12">
   <si>
     <r>
       <t>feature</t>
@@ -127,37 +127,13 @@
     <t>RSV</t>
   </si>
   <si>
-    <t>respiratory syncytial virus, specific</t>
-  </si>
-  <si>
-    <t>Respiratorisches Syncytial-Virus, spezifisch</t>
-  </si>
-  <si>
-    <t>specific RSV-ICD-10 codes</t>
-  </si>
-  <si>
-    <t>respiratory syncytial virus, unspecific</t>
-  </si>
-  <si>
-    <t>Respiratorisches Syncytial-Virus, unspezifisch</t>
-  </si>
-  <si>
-    <t>unspecific ALRI-ICD-10 codes AND &lt;=2 years old</t>
-  </si>
-  <si>
     <t>GI</t>
   </si>
   <si>
-    <t>non-bleeding unspecific gastrointestinal infections</t>
+    <t/>
   </si>
   <si>
-    <t>nicht-blutige unspezifische gastrointestinale Infektionen</t>
-  </si>
-  <si>
-    <t>MTS/CEDIS + gi-specific ICD (non bloody)</t>
-  </si>
-  <si>
-    <t/>
+    <t>Lorem Ipsum</t>
   </si>
 </sst>
 </file>
@@ -281,7 +257,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -300,9 +276,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -319,7 +292,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -623,16 +596,16 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:AD16"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.28515625" style="12" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.7109375" style="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.5703125" style="13" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="39.28515625" style="12" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="76.5703125" style="12" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="60.5703125" style="12" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="82.5703125" style="14" bestFit="1" customWidth="1"/>
-    <col min="8" max="30" width="13.5703125" style="12" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.28515625" style="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.7109375" style="11" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.5703125" style="12" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="39.28515625" style="11" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="76.5703125" style="11" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="60.5703125" style="11" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="82.5703125" style="13" bestFit="1" customWidth="1"/>
+    <col min="8" max="30" width="13.5703125" style="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:30" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -696,12 +669,12 @@
         <v>feat_syndrome_RSV_01</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="G2" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" s="11" t="s">
         <v>11</v>
       </c>
       <c r="H2" s="5"/>
@@ -742,14 +715,14 @@
         <f>A3&amp;"_"&amp;B3&amp;"_"&amp;TEXT(C3,"00")</f>
         <v>feat_syndrome_RSV_02</v>
       </c>
-      <c r="E3" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G3" s="8" t="s">
-        <v>14</v>
+      <c r="E3" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>11</v>
       </c>
       <c r="H3" s="5"/>
       <c r="I3" s="5"/>
@@ -780,7 +753,7 @@
         <v>7</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="C4" s="6">
         <v>1</v>
@@ -789,14 +762,14 @@
         <f>A4&amp;"_"&amp;B4&amp;"_"&amp;TEXT(C4,"00")</f>
         <v>feat_syndrome_GI_01</v>
       </c>
-      <c r="E4" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G4" s="8" t="s">
-        <v>18</v>
+      <c r="E4" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>11</v>
       </c>
       <c r="H4" s="5"/>
       <c r="I4" s="5"/>
@@ -823,24 +796,24 @@
       <c r="AD4" s="5"/>
     </row>
     <row r="5" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A5" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>19</v>
+      <c r="A5" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>10</v>
       </c>
       <c r="C5" s="6"/>
-      <c r="D5" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E5" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F5" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="G5" s="10" t="s">
-        <v>19</v>
+      <c r="D5" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>10</v>
       </c>
       <c r="H5" s="5"/>
       <c r="I5" s="5"/>
@@ -867,24 +840,24 @@
       <c r="AD5" s="5"/>
     </row>
     <row r="6" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A6" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>19</v>
+      <c r="A6" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>10</v>
       </c>
       <c r="C6" s="6"/>
-      <c r="D6" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="G6" s="10" t="s">
-        <v>19</v>
+      <c r="D6" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>10</v>
       </c>
       <c r="H6" s="5"/>
       <c r="I6" s="5"/>
@@ -911,24 +884,24 @@
       <c r="AD6" s="5"/>
     </row>
     <row r="7" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A7" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>19</v>
+      <c r="A7" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>10</v>
       </c>
       <c r="C7" s="6"/>
-      <c r="D7" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F7" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="G7" s="10" t="s">
-        <v>19</v>
+      <c r="D7" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>10</v>
       </c>
       <c r="H7" s="5"/>
       <c r="I7" s="5"/>
@@ -955,24 +928,24 @@
       <c r="AD7" s="5"/>
     </row>
     <row r="8" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A8" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>19</v>
+      <c r="A8" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>10</v>
       </c>
       <c r="C8" s="6"/>
-      <c r="D8" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E8" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F8" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="G8" s="10" t="s">
-        <v>19</v>
+      <c r="D8" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>10</v>
       </c>
       <c r="H8" s="5"/>
       <c r="I8" s="5"/>
@@ -999,24 +972,24 @@
       <c r="AD8" s="5"/>
     </row>
     <row r="9" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A9" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>19</v>
+      <c r="A9" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>10</v>
       </c>
       <c r="C9" s="6"/>
-      <c r="D9" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E9" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F9" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="G9" s="10" t="s">
-        <v>19</v>
+      <c r="D9" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G9" s="9" t="s">
+        <v>10</v>
       </c>
       <c r="H9" s="5"/>
       <c r="I9" s="5"/>
@@ -1043,24 +1016,24 @@
       <c r="AD9" s="5"/>
     </row>
     <row r="10" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A10" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>19</v>
+      <c r="A10" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>10</v>
       </c>
       <c r="C10" s="6"/>
-      <c r="D10" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F10" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="G10" s="10" t="s">
-        <v>19</v>
+      <c r="D10" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G10" s="9" t="s">
+        <v>10</v>
       </c>
       <c r="H10" s="5"/>
       <c r="I10" s="5"/>
@@ -1087,24 +1060,24 @@
       <c r="AD10" s="5"/>
     </row>
     <row r="11" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A11" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>19</v>
+      <c r="A11" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>10</v>
       </c>
       <c r="C11" s="6"/>
-      <c r="D11" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E11" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F11" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="G11" s="10" t="s">
-        <v>19</v>
+      <c r="D11" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G11" s="9" t="s">
+        <v>10</v>
       </c>
       <c r="H11" s="5"/>
       <c r="I11" s="5"/>
@@ -1131,24 +1104,24 @@
       <c r="AD11" s="5"/>
     </row>
     <row r="12" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A12" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>19</v>
+      <c r="A12" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>10</v>
       </c>
       <c r="C12" s="6"/>
-      <c r="D12" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E12" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F12" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="G12" s="10" t="s">
-        <v>19</v>
+      <c r="D12" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G12" s="9" t="s">
+        <v>10</v>
       </c>
       <c r="H12" s="5"/>
       <c r="I12" s="5"/>
@@ -1175,24 +1148,24 @@
       <c r="AD12" s="5"/>
     </row>
     <row r="13" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A13" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>19</v>
+      <c r="A13" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>10</v>
       </c>
       <c r="C13" s="6"/>
-      <c r="D13" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E13" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F13" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="G13" s="10" t="s">
-        <v>19</v>
+      <c r="D13" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G13" s="9" t="s">
+        <v>10</v>
       </c>
       <c r="H13" s="5"/>
       <c r="I13" s="5"/>
@@ -1219,24 +1192,24 @@
       <c r="AD13" s="5"/>
     </row>
     <row r="14" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A14" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B14" s="9" t="s">
-        <v>19</v>
+      <c r="A14" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>10</v>
       </c>
       <c r="C14" s="6"/>
-      <c r="D14" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E14" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F14" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="G14" s="10" t="s">
-        <v>19</v>
+      <c r="D14" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G14" s="9" t="s">
+        <v>10</v>
       </c>
       <c r="H14" s="5"/>
       <c r="I14" s="5"/>
@@ -1263,24 +1236,24 @@
       <c r="AD14" s="5"/>
     </row>
     <row r="15" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A15" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B15" s="9" t="s">
-        <v>19</v>
+      <c r="A15" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>10</v>
       </c>
       <c r="C15" s="6"/>
-      <c r="D15" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E15" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F15" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="G15" s="10" t="s">
-        <v>19</v>
+      <c r="D15" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G15" s="9" t="s">
+        <v>10</v>
       </c>
       <c r="H15" s="5"/>
       <c r="I15" s="5"/>
@@ -1307,24 +1280,24 @@
       <c r="AD15" s="5"/>
     </row>
     <row r="16" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A16" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B16" s="9" t="s">
-        <v>19</v>
+      <c r="A16" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>10</v>
       </c>
       <c r="C16" s="6"/>
-      <c r="D16" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E16" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F16" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="G16" s="11" t="s">
-        <v>19</v>
+      <c r="D16" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G16" s="10" t="s">
+        <v>10</v>
       </c>
       <c r="H16" s="5"/>
       <c r="I16" s="5"/>

</xml_diff>